<commit_message>
Finalize v7 baselines: add docs + play-tested workbooks
Adds BASELINE_v7_ALL_CONFIGS.md (reference notes) and
BASELINE_LINEAGE_v4_to_v7.md (baseline genealogy). Replaces the three
BASELINE_v7_*.xlsx with the play-tested workbooks; data is identical to the
generated set (every financial figure matches), differing only in the display
starting year (2026 vs 2025).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KByPnmZqFHAjC6MDpsfvdF
</commit_message>
<xml_diff>
--- a/baselines/BASELINE_v7_WC.xlsx
+++ b/baselines/BASELINE_v7_WC.xlsx
@@ -408,13 +408,13 @@
         <v>Metric</v>
       </c>
       <c r="C1" t="str">
-        <v>Year 1 / 2025</v>
+        <v>Year 1 / 2026</v>
       </c>
       <c r="D1" t="str">
-        <v>Year 2 / 2026</v>
+        <v>Year 2 / 2027</v>
       </c>
       <c r="E1" t="str">
-        <v>Year 3 / 2027</v>
+        <v>Year 3 / 2028</v>
       </c>
     </row>
     <row r="2">
@@ -442,13 +442,13 @@
         <v>Calendar Year</v>
       </c>
       <c r="C3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D3">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E3">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="4">
@@ -1819,13 +1819,13 @@
         <v>Excess Capital Ratio</v>
       </c>
       <c r="C84">
-        <v>1.3109577750035035</v>
+        <v>1.310957775003503</v>
       </c>
       <c r="D84">
-        <v>0.9955599802755499</v>
+        <v>0.9955599802755495</v>
       </c>
       <c r="E84">
-        <v>1.0489436262512364</v>
+        <v>1.0489436262512362</v>
       </c>
     </row>
     <row r="85">
@@ -1864,13 +1864,13 @@
         <v>Metric</v>
       </c>
       <c r="C1" t="str">
-        <v>Year 1 / 2025</v>
+        <v>Year 1 / 2026</v>
       </c>
       <c r="D1" t="str">
-        <v>Year 2 / 2026</v>
+        <v>Year 2 / 2027</v>
       </c>
       <c r="E1" t="str">
-        <v>Year 3 / 2027</v>
+        <v>Year 3 / 2028</v>
       </c>
     </row>
     <row r="2">
@@ -1898,13 +1898,13 @@
         <v>Calendar Year</v>
       </c>
       <c r="C3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D3">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E3">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="4">
@@ -3309,13 +3309,13 @@
         <v>Excess Capital Ratio</v>
       </c>
       <c r="C86">
-        <v>1.3109577750035035</v>
+        <v>1.310957775003503</v>
       </c>
       <c r="D86">
-        <v>0.9955599802755499</v>
+        <v>0.9955599802755495</v>
       </c>
       <c r="E86">
-        <v>1.0489436262512364</v>
+        <v>1.0489436262512362</v>
       </c>
     </row>
     <row r="87">

</xml_diff>